<commit_message>
feat: Update NAV data and metal prices; modify finance data file
</commit_message>
<xml_diff>
--- a/sample_finance_data.xlsx
+++ b/sample_finance_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\data\tools\personal\port\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0495C6E4-BBD6-4070-8EBE-3D63B2782842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E454E43F-5240-4E29-BF37-4222FD74AE16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="42">
   <si>
     <t>FundName</t>
   </si>
@@ -133,6 +133,24 @@
   </si>
   <si>
     <t>UTI Nifty 50 Index Fund Direct Growth</t>
+  </si>
+  <si>
+    <t>Motilal Oswal ELSS Tax Saver Fund Direct Growth</t>
+  </si>
+  <si>
+    <t>Parag Parikh Flexi Cap Fund Direct Growth</t>
+  </si>
+  <si>
+    <t>Navi Nifty Smallcap250 Momentum Quality 100 Index Fund Direct Growth</t>
+  </si>
+  <si>
+    <t>Sundaram Arbitrage Fund Direct Growth</t>
+  </si>
+  <si>
+    <t>Nippon India Nifty IT Index Fund Direct Growth</t>
+  </si>
+  <si>
+    <t>Kotak Nifty Next 50 Index Fund Direct Growth</t>
   </si>
 </sst>
 </file>
@@ -472,10 +490,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="67.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
@@ -496,10 +514,76 @@
         <v>35</v>
       </c>
       <c r="B2">
-        <v>172.113</v>
+        <v>255.56200000000001</v>
       </c>
       <c r="C2">
         <v>120716</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3">
+        <v>749.70799999999997</v>
+      </c>
+      <c r="C3">
+        <v>148745</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4">
+        <v>3147.7440000000001</v>
+      </c>
+      <c r="C4">
+        <v>153362</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5">
+        <v>3342.4929999999999</v>
+      </c>
+      <c r="C5">
+        <v>152392</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6">
+        <v>865.74599999999998</v>
+      </c>
+      <c r="C6">
+        <v>133386</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7">
+        <v>465.76900000000001</v>
+      </c>
+      <c r="C7">
+        <v>122639</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8">
+        <v>1671.6310000000001</v>
+      </c>
+      <c r="C8">
+        <v>149550</v>
       </c>
     </row>
   </sheetData>
@@ -545,6 +629,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -599,6 +688,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -673,6 +768,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>